<commit_message>
feat: append TM schema ID 1944
</commit_message>
<xml_diff>
--- a/template/Bank_TM_ReportNormId.xlsx
+++ b/template/Bank_TM_ReportNormId.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1387" uniqueCount="540">
   <si>
     <t>ReportNormId</t>
   </si>
@@ -1636,6 +1636,9 @@
   </si>
   <si>
     <t>Rủi ro thanh khoản - Tổng</t>
+  </si>
+  <si>
+    <t>Cho vay giao dịch ký quỹ và ứng trước tiền bán chứng khoán</t>
   </si>
 </sst>
 </file>
@@ -2010,7 +2013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1385"/>
+  <dimension ref="A1:C1386"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="100.625" bestFit="1" customWidth="1"/>
@@ -17248,6 +17251,17 @@
         <v>531</v>
       </c>
     </row>
+    <row r="1386" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A1386" s="1">
+        <v>1384</v>
+      </c>
+      <c r="B1386">
+        <v>1944</v>
+      </c>
+      <c r="C1386" t="s">
+        <v>539</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>